<commit_message>
Anteproyectos: segundo proyecto (PEH Tecate) y nuevo acomodo de la hoja RTA
- Excel con el avance programado del primer proyecto y el segundo
  proyecto (PEH Tecate, Equipamiento Hidroeléctrico).
- La hoja RTA ahora puede tener la fila de grupos arriba
  ("Identificadores", "Especificaciones del sistema"...) y "No." y
  "Proyecto" en la fila de encabezados; el acomodo anterior sigue
  funcionando (con prueba).
- KML: el punto "TECATE" se llama "PEH Tecate", igual que el proyecto,
  para que salga en el mapa.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01APiq7bAy76yveceNZKtsYf
</commit_message>
<xml_diff>
--- a/cartera-anteproyectos/data/datos_anteproyectos.xlsx
+++ b/cartera-anteproyectos/data/datos_anteproyectos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CN594\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E6622F0-0F7F-496F-BD7C-7F4DAD39450E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F2C11E4-E5DB-49E8-BCB4-279A5BB3DC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="839" activeTab="4" xr2:uid="{F77216BA-A0B8-4B6C-9AC8-5CF7CF39AEC5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="839" xr2:uid="{F77216BA-A0B8-4B6C-9AC8-5CF7CF39AEC5}"/>
   </bookViews>
   <sheets>
     <sheet name="PRES" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="145">
   <si>
     <t>PFV Isla Cayacal (Petacalco)</t>
   </si>
@@ -208,20 +208,9 @@
     <t>Se ha definido una potencia preliminar de 16 Mwac</t>
   </si>
   <si>
-    <t>Se estudiaron 5 alternativas. En proceso informe.</t>
-  </si>
-  <si>
-    <t>NOTA (2.4)</t>
-  </si>
-  <si>
     <t>NOTA TOTAL</t>
   </si>
   <si>
-    <t>•	Los resultados obtenidos a la fecha muestran un sobrecosto aproximado del 20%, debido al movimiento de tierras necesario para la disposición de los paneles fotovoltaicos.
-•	Se preparó presentación ejecutiva de la reconfiguración del proyecto considerando las condiciones del sitio Cayacal con depósitos de ceniza. Está en proceso el informe respectivo.
-•	Se plantea 2da visita con personal del área ambiental.</t>
-  </si>
-  <si>
     <t>Imagen</t>
   </si>
   <si>
@@ -333,9 +322,6 @@
     <t>Subestación Lázaro Cárdenas Potencia</t>
   </si>
   <si>
-    <t xml:space="preserve">Conexión en el nodo 01LCP-230 de la SE Lázaro Cárdenas Potencia del sistema de transmisión nacional/regional. </t>
-  </si>
-  <si>
     <t>Alta Confiabilidad</t>
   </si>
   <si>
@@ -346,6 +332,176 @@
   </si>
   <si>
     <t>Punto de Interconexión (POI)</t>
+  </si>
+  <si>
+    <t>•	Se estudian cuatro alternativas con diferentes soluciones para la conformación del predio considerando los depósitos de ceniza. Está en proceso el informe respectivo.
+•	Se coordinará 2da visita técnica (diciembre 2026) en conjunto con la ASIPONA (Administración del Sistema Portuario Nacional), a fin de validar las condiciones y consideraciones ambientales y sociales en la zona del proyecto.</t>
+  </si>
+  <si>
+    <t>Nivel de estudio</t>
+  </si>
+  <si>
+    <t>Prefactibilidad</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>PEH Tecate</t>
+  </si>
+  <si>
+    <t>Equipamiento Hidroeléctrico</t>
+  </si>
+  <si>
+    <t>Tecate, Baja California</t>
+  </si>
+  <si>
+    <t>data/IMAGENES/TECATE.jpg</t>
+  </si>
+  <si>
+    <t>El Proyecto de Equipamiento Hidroeléctrico aprovecha las descargas del Acueducto Río Colorado – Tijuana mediante la incorporación de una derivación que conecta con un tanque puesta a presión y que mediante una tubería a presión conecta con la casa de máquinas que se ubica en un afluente innominado para aprovechar una carga bruta de 580 m para generar energía eléctrica y, posteriormente, descargar en la Presa El Carrizo.
+El diseño del equipamiento considera las condiciones actuales de operación del Acueducto con una operación continua que abastece de agua a la ciudad de Tijuana, Baja California, aportando energía al Sistema Eléctrico Tijuana – Ensenada. Las obras consideradas en el proyecto son:
+1. Tubería a presión
+2. Tanque puesta a presión
+3. Casa de Máquinas
+4. Subestación elevadora
+5. Interconexión</t>
+  </si>
+  <si>
+    <t>Minimización del trazado para reducir pérdidas técnicas y costos de inversión en conductor y contar con capacidad Enel NODO</t>
+  </si>
+  <si>
+    <t>Celosía metálica, altura 30-35 m</t>
+  </si>
+  <si>
+    <t>28 Unid.</t>
+  </si>
+  <si>
+    <t>Subestación La Herradura</t>
+  </si>
+  <si>
+    <t>Conexión en el nodo 07-HRA-69 del sistema de transmisión nacional/regional.</t>
+  </si>
+  <si>
+    <t>Conexión en el nodo 01LCP-230 de la SE Lázaro Cárdenas Potencia del sistema de transmisión nacional/regional</t>
+  </si>
+  <si>
+    <t>Identificadores</t>
+  </si>
+  <si>
+    <t>Potencia Instalada [MW]</t>
+  </si>
+  <si>
+    <t>19.4</t>
+  </si>
+  <si>
+    <t>Generación media anual [GWh]</t>
+  </si>
+  <si>
+    <t>170</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>Número de turbinas [#]</t>
+  </si>
+  <si>
+    <t>Tipo de turbina</t>
+  </si>
+  <si>
+    <t>Pelton</t>
+  </si>
+  <si>
+    <t>Consumo específico [m3/kWh]</t>
+  </si>
+  <si>
+    <t>0.74</t>
+  </si>
+  <si>
+    <t>Gasto de diseño [m3/s]</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Carga bruta [m]</t>
+  </si>
+  <si>
+    <t>580</t>
+  </si>
+  <si>
+    <t>Volumen Útil</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Nodo de Interconexión</t>
+  </si>
+  <si>
+    <t>S.E. La Herradura</t>
+  </si>
+  <si>
+    <t>1 Certidumbre Social, Ambiental, Tenencia de la tierra e Hídrica</t>
+  </si>
+  <si>
+    <t>1.1 Análisis de la disponibilidad y factibilidad del uso del recurso hídrico.</t>
+  </si>
+  <si>
+    <t>1.2 Gestión con la CEA de BC y la CONAGUA entorno a la concesión de agua.</t>
+  </si>
+  <si>
+    <t>1.3 Tenencia de la tierra</t>
+  </si>
+  <si>
+    <t>1.4 Diagnóstico social preliminar.</t>
+  </si>
+  <si>
+    <t>1.5 Diagnóstico ambiental preliminar.</t>
+  </si>
+  <si>
+    <t>1.6 Diagnóstico arqueológico preliminar.</t>
+  </si>
+  <si>
+    <t>1.7 Análisis FODA.</t>
+  </si>
+  <si>
+    <t>2 Desarrollo de Ingeniería (Anteproyecto)</t>
+  </si>
+  <si>
+    <t>2.1 Visita técnica al sitio del proyecto.</t>
+  </si>
+  <si>
+    <t>2.2 Levantamiento topográfico LiDAR con Dron.</t>
+  </si>
+  <si>
+    <t>2.3 Análisis de la operación del Acueducto y Estudio hidrológico.</t>
+  </si>
+  <si>
+    <t>2.4 Planteamiento de obras principales (toma, conducción a presión, casa de máquinas)</t>
+  </si>
+  <si>
+    <t>2.5 Obras complementarias requeridas.</t>
+  </si>
+  <si>
+    <t>2.6 Estimación preliminar de CAPEX , OPEX y programa de obra.</t>
+  </si>
+  <si>
+    <t>•	El 18 de septiembre la Secretaría para el Manejo, Saneamiento y Protección del Agua (SEPROA) entregó a la CPEL información técnica del acueducto. Esta información muestra incertidumbre en la disponibilidad del agua a largo plazo para el aprovechamiento del proyecto. 
+•	Se gestionará visita técnica en noviembre, se llevará a cabo posterior a la presentación del proyecto a la SEPROA (Secretaría para el Manejo, Saneamiento y Protección del Agua de Baja California).</t>
+  </si>
+  <si>
+    <t>•	La disponibilidad no es la prevista inicialmente</t>
+  </si>
+  <si>
+    <t>NOTA (1.1)</t>
+  </si>
+  <si>
+    <t>•	Se recabó en catastro municipal plano general de propietarios</t>
+  </si>
+  <si>
+    <t>NOTA (1.3)</t>
   </si>
 </sst>
 </file>
@@ -414,7 +570,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="52">
     <border>
       <left/>
       <right/>
@@ -449,136 +605,105 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="hair">
         <color indexed="64"/>
       </left>
-      <right/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="hair">
         <color indexed="64"/>
       </right>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color indexed="64"/>
-      </left>
-      <right style="hair">
-        <color indexed="64"/>
-      </right>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color indexed="64"/>
-      </left>
-      <right style="hair">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="hair">
-        <color indexed="64"/>
-      </right>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="hair">
-        <color indexed="64"/>
-      </right>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="hair">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="hair">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="hair">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top/>
       <bottom style="medium">
         <color indexed="64"/>
@@ -935,6 +1060,169 @@
       </right>
       <top/>
       <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="hair">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -944,132 +1232,176 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="47" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="41" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="40" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="46" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1406,50 +1738,78 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7582F8E4-5871-4CE4-85C7-5CB4D3DD57AE}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="27" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="1"/>
-    <col min="7" max="7" width="11.42578125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.42578125" style="1"/>
+    <col min="3" max="3" width="26.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" style="1"/>
+    <col min="8" max="8" width="11.42578125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="70" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="71" t="s">
+      <c r="C1" s="36" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="71" t="s">
+      <c r="E1" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="72" t="s">
-        <v>53</v>
+      <c r="F1" s="37" t="s">
+        <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="68">
+    <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="33">
         <v>1</v>
       </c>
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="69" t="s">
+      <c r="C2" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="69" t="s">
+      <c r="E2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="73" t="s">
-        <v>92</v>
+      <c r="F2" s="38" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="E3" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="F3" s="38" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1462,9 +1822,112 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="31" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="E1" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="H1" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="I1" s="31" t="s">
+        <v>117</v>
+      </c>
+      <c r="J1" s="31" t="s">
+        <v>119</v>
+      </c>
+      <c r="K1" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="L1" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="M1" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="N1" s="32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2" s="34" t="s">
+        <v>110</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="G2" s="34" t="s">
+        <v>114</v>
+      </c>
+      <c r="H2" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="I2" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="J2" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="K2" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="L2" s="34" t="s">
+        <v>124</v>
+      </c>
+      <c r="M2" s="8">
+        <v>54.5</v>
+      </c>
+      <c r="N2" s="9">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1474,9 +1937,215 @@
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="19" width="15.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>127</v>
+      </c>
+      <c r="H1" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="I1" s="21" t="s">
+        <v>129</v>
+      </c>
+      <c r="J1" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="K1" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="L1" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="M1" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="N1" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="O1" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="P1" s="24" t="s">
+        <v>136</v>
+      </c>
+      <c r="Q1" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="R1" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="S1" s="24" t="s">
+        <v>139</v>
+      </c>
+      <c r="T1" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="U1" s="43" t="s">
+        <v>142</v>
+      </c>
+      <c r="V1" s="22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A2" s="67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="69" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0.33</v>
+      </c>
+      <c r="E2" s="3">
+        <v>0.31</v>
+      </c>
+      <c r="F2" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="G2" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="J2" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="K2" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="L2" s="3">
+        <v>0</v>
+      </c>
+      <c r="M2" s="3">
+        <v>0.34</v>
+      </c>
+      <c r="N2" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="O2" s="3">
+        <v>0</v>
+      </c>
+      <c r="P2" s="25">
+        <v>0.7</v>
+      </c>
+      <c r="Q2" s="25">
+        <v>0.65</v>
+      </c>
+      <c r="R2" s="25">
+        <v>0.2</v>
+      </c>
+      <c r="S2" s="25">
+        <v>0.2</v>
+      </c>
+      <c r="T2" s="42" t="s">
+        <v>140</v>
+      </c>
+      <c r="U2" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="V2" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="68"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="23">
+        <v>0.47</v>
+      </c>
+      <c r="E3" s="23">
+        <v>0.61</v>
+      </c>
+      <c r="F3" s="23">
+        <v>0.75</v>
+      </c>
+      <c r="G3" s="23">
+        <v>0.63</v>
+      </c>
+      <c r="H3" s="23">
+        <v>0.75</v>
+      </c>
+      <c r="I3" s="23">
+        <v>0.69</v>
+      </c>
+      <c r="J3" s="23">
+        <v>0.69</v>
+      </c>
+      <c r="K3" s="23">
+        <v>0.75</v>
+      </c>
+      <c r="L3" s="23">
+        <v>0</v>
+      </c>
+      <c r="M3" s="23">
+        <v>0.33</v>
+      </c>
+      <c r="N3" s="23">
+        <v>0.17</v>
+      </c>
+      <c r="O3" s="23">
+        <v>0</v>
+      </c>
+      <c r="P3" s="26">
+        <v>0.75</v>
+      </c>
+      <c r="Q3" s="26">
+        <v>0.63</v>
+      </c>
+      <c r="R3" s="26">
+        <v>0.44</v>
+      </c>
+      <c r="S3" s="26">
+        <v>0</v>
+      </c>
+      <c r="T3" s="29"/>
+      <c r="U3" s="13"/>
+      <c r="V3" s="14"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1507,7 +2176,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45D77318-4E74-4035-A05D-AC6B6DDDAC7C}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
@@ -1516,25 +2185,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="65" t="s">
+      <c r="B1" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="74" t="s">
+      <c r="C1" s="39" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="255.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="75">
+    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="40">
         <v>1</v>
       </c>
-      <c r="B2" s="76" t="s">
+      <c r="B2" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="77" t="s">
+      <c r="C2" s="44" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" s="34" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1544,7 +2224,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37E307FA-5186-457C-8CE8-B07656929254}">
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
@@ -1552,7 +2232,7 @@
     <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.28515625" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.7109375" bestFit="1" customWidth="1"/>
@@ -1563,243 +2243,348 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="86" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="87"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
+      <c r="I1" s="87"/>
+      <c r="J1" s="87"/>
+      <c r="K1" s="87"/>
+      <c r="L1" s="87"/>
+      <c r="M1" s="87"/>
+      <c r="N1" s="87"/>
+      <c r="O1" s="87"/>
+      <c r="P1" s="87"/>
+      <c r="Q1" s="88"/>
+    </row>
+    <row r="2" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="77" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" s="78"/>
+      <c r="C2" s="77" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="85"/>
+      <c r="E2" s="85"/>
+      <c r="F2" s="85"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="77" t="s">
+        <v>61</v>
+      </c>
+      <c r="J2" s="85"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="77" t="s">
+        <v>89</v>
+      </c>
+      <c r="M2" s="85"/>
+      <c r="N2" s="89"/>
+      <c r="O2" s="77" t="s">
+        <v>90</v>
+      </c>
+      <c r="P2" s="85"/>
+      <c r="Q2" s="78"/>
+    </row>
+    <row r="3" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="65" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="66" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="60" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="61" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" s="61" t="s">
+        <v>52</v>
+      </c>
+      <c r="F3" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="G3" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" s="62" t="s">
+        <v>54</v>
+      </c>
+      <c r="I3" s="63" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="61" t="s">
+        <v>63</v>
+      </c>
+      <c r="K3" s="62" t="s">
+        <v>64</v>
+      </c>
+      <c r="L3" s="63" t="s">
+        <v>80</v>
+      </c>
+      <c r="M3" s="61" t="s">
+        <v>81</v>
+      </c>
+      <c r="N3" s="64" t="s">
+        <v>83</v>
+      </c>
+      <c r="O3" s="63" t="s">
+        <v>84</v>
+      </c>
+      <c r="P3" s="61" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q3" s="62" t="s">
         <v>85</v>
-      </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="45"/>
-      <c r="N1" s="45"/>
-      <c r="O1" s="45"/>
-      <c r="P1" s="45"/>
-      <c r="Q1" s="46"/>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="38" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="39" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="40" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="40" t="s">
-        <v>64</v>
-      </c>
-      <c r="J2" s="41"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="40" t="s">
-        <v>93</v>
-      </c>
-      <c r="M2" s="41"/>
-      <c r="N2" s="43"/>
-      <c r="O2" s="40" t="s">
-        <v>94</v>
-      </c>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="42"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="13">
-        <v>1</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="I3" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="K3" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="L3" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="M3" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="N3" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="O3" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="P3" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q3" s="14" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="25">
+      <c r="A4" s="79">
+        <v>1</v>
+      </c>
+      <c r="B4" s="82" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="55">
         <v>115</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="56">
         <v>16.3</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="56" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4" s="56">
+        <v>0.2</v>
+      </c>
+      <c r="G4" s="56" t="s">
+        <v>59</v>
+      </c>
+      <c r="H4" s="57" t="s">
         <v>60</v>
       </c>
-      <c r="F4" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="H4" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="I4" s="30" t="s">
+      <c r="I4" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L4" s="58" t="s">
         <v>68</v>
       </c>
-      <c r="J4" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="K4" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="L4" s="32" t="s">
-        <v>71</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="N4" s="35" t="s">
-        <v>79</v>
-      </c>
-      <c r="O4" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="P4" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="Q4" s="16" t="s">
-        <v>91</v>
+      <c r="M4" s="56" t="s">
+        <v>72</v>
+      </c>
+      <c r="N4" s="59" t="s">
+        <v>76</v>
+      </c>
+      <c r="O4" s="58" t="s">
+        <v>86</v>
+      </c>
+      <c r="P4" s="56" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q4" s="57" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="15"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="27"/>
-      <c r="L5" s="25" t="s">
-        <v>72</v>
+      <c r="A5" s="80"/>
+      <c r="B5" s="83"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="11"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="10" t="s">
+        <v>69</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="N5" s="36" t="s">
-        <v>80</v>
-      </c>
-      <c r="O5" s="26"/>
-      <c r="P5" s="17"/>
-      <c r="Q5" s="27"/>
+        <v>73</v>
+      </c>
+      <c r="N5" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="O5" s="11"/>
+      <c r="Q5" s="12"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="25" t="s">
-        <v>73</v>
+      <c r="A6" s="80"/>
+      <c r="B6" s="83"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="11"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="10" t="s">
+        <v>70</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="N6" s="36" t="s">
-        <v>81</v>
-      </c>
-      <c r="O6" s="26"/>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="27"/>
+        <v>74</v>
+      </c>
+      <c r="N6" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="O6" s="11"/>
+      <c r="Q6" s="12"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="19"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="29"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="29"/>
-      <c r="L7" s="33" t="s">
+      <c r="A7" s="81"/>
+      <c r="B7" s="84"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="N7" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="O7" s="13"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="14"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="74" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8" s="71" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" s="50">
+        <v>115</v>
+      </c>
+      <c r="D8" s="51">
+        <v>19</v>
+      </c>
+      <c r="E8" s="51" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="51">
+        <v>11</v>
+      </c>
+      <c r="G8" s="51" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" s="52" t="s">
+        <v>60</v>
+      </c>
+      <c r="I8" s="47" t="s">
+        <v>100</v>
+      </c>
+      <c r="J8" s="48" t="s">
+        <v>66</v>
+      </c>
+      <c r="K8" s="49" t="s">
+        <v>67</v>
+      </c>
+      <c r="L8" s="53" t="s">
+        <v>68</v>
+      </c>
+      <c r="M8" s="45" t="s">
+        <v>101</v>
+      </c>
+      <c r="N8" s="46" t="s">
+        <v>102</v>
+      </c>
+      <c r="O8" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="P8" s="48" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q8" s="49" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="75"/>
+      <c r="B9" s="72"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="11"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="N9" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="O9" s="11"/>
+      <c r="Q9" s="12"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="75"/>
+      <c r="B10" s="72"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="11"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="M10" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="M7" s="22" t="s">
+      <c r="N10" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="N7" s="37" t="s">
-        <v>82</v>
-      </c>
-      <c r="O7" s="28"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="29"/>
+      <c r="O10" s="11"/>
+      <c r="Q10" s="12"/>
+    </row>
+    <row r="11" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="76"/>
+      <c r="B11" s="73"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="54" t="s">
+        <v>71</v>
+      </c>
+      <c r="M11" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="N11" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="O11" s="13"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="10">
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="C2:H2"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="L2:N2"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A4:A7"/>
+    <mergeCell ref="B4:B7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1832,102 +2617,102 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="65" t="s">
+      <c r="B1" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="65" t="s">
+      <c r="C1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="65" t="s">
+      <c r="D1" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="65" t="s">
+      <c r="E1" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="65" t="s">
+      <c r="F1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="65" t="s">
+      <c r="G1" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="65" t="s">
+      <c r="H1" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="65" t="s">
+      <c r="I1" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="65" t="s">
+      <c r="J1" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="66" t="s">
+      <c r="K1" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="L1" s="66" t="s">
+      <c r="L1" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="66" t="s">
+      <c r="M1" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="66" t="s">
+      <c r="N1" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="66" t="s">
+      <c r="O1" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="P1" s="67" t="s">
+      <c r="P1" s="32" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="68">
+      <c r="A2" s="33">
         <v>1</v>
       </c>
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="69">
+      <c r="C2" s="34">
         <v>19.7</v>
       </c>
-      <c r="D2" s="69">
+      <c r="D2" s="34">
         <v>16.3</v>
       </c>
-      <c r="E2" s="69">
+      <c r="E2" s="34">
         <v>21</v>
       </c>
-      <c r="F2" s="69">
+      <c r="F2" s="34">
         <v>36.6</v>
       </c>
-      <c r="G2" s="69">
+      <c r="G2" s="34">
         <v>5.8</v>
       </c>
-      <c r="H2" s="69">
+      <c r="H2" s="34">
         <v>650</v>
       </c>
-      <c r="I2" s="69">
+      <c r="I2" s="34">
         <v>24.06</v>
       </c>
-      <c r="J2" s="69" t="s">
+      <c r="J2" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="22">
+      <c r="K2" s="8">
         <v>1</v>
       </c>
-      <c r="L2" s="22" t="s">
+      <c r="L2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="22" t="s">
+      <c r="M2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="N2" s="22" t="s">
+      <c r="N2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="22" t="s">
+      <c r="O2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="23" t="s">
+      <c r="P2" s="9" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1944,106 +2729,103 @@
   <sheetPr>
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="39.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="53.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="38.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="40.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="51.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="23.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="20" width="39" style="4" customWidth="1"/>
-    <col min="21" max="16384" width="11.42578125" style="4"/>
+    <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="53.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="40.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="51.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="39" customWidth="1"/>
+    <col min="19" max="19" width="46.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="48" t="s">
+      <c r="C1" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="48" t="s">
+      <c r="D1" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="48" t="s">
+      <c r="E1" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="48" t="s">
+      <c r="F1" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="48" t="s">
+      <c r="G1" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="48" t="s">
+      <c r="H1" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="I1" s="48" t="s">
+      <c r="I1" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="J1" s="48" t="s">
+      <c r="J1" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="K1" s="48" t="s">
+      <c r="K1" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="L1" s="48" t="s">
+      <c r="L1" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="M1" s="48" t="s">
+      <c r="M1" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="N1" s="48" t="s">
+      <c r="N1" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="O1" s="48" t="s">
+      <c r="O1" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="P1" s="56" t="s">
+      <c r="P1" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="Q1" s="61" t="s">
-        <v>51</v>
-      </c>
-      <c r="R1" s="59" t="s">
+      <c r="Q1" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="R1" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="S1" s="49" t="s">
+      <c r="S1" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="T1" s="50" t="s">
-        <v>50</v>
-      </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A2" s="13">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" s="92">
         <v>1</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="90" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>38</v>
       </c>
       <c r="D2" s="3">
-        <v>0.57999999999999996</v>
+        <v>0.59</v>
       </c>
       <c r="E2" s="3">
-        <v>0.56000000000000005</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="F2" s="3">
         <v>0.5</v>
@@ -2055,10 +2837,10 @@
         <v>0.5</v>
       </c>
       <c r="I2" s="3">
-        <v>0.6</v>
+        <v>0.64</v>
       </c>
       <c r="J2" s="3">
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="K2" s="3">
         <v>1</v>
@@ -2067,7 +2849,7 @@
         <v>1</v>
       </c>
       <c r="M2" s="3">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="N2" s="3">
         <v>0.15</v>
@@ -2075,71 +2857,67 @@
       <c r="O2" s="3">
         <v>0.3</v>
       </c>
-      <c r="P2" s="57">
+      <c r="P2" s="25">
         <v>0.5</v>
       </c>
-      <c r="Q2" s="62" t="s">
-        <v>52</v>
-      </c>
-      <c r="R2" s="60" t="s">
+      <c r="Q2" s="42" t="s">
+        <v>91</v>
+      </c>
+      <c r="R2" s="10" t="s">
         <v>46</v>
       </c>
       <c r="S2" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="T2" s="51" t="s">
-        <v>49</v>
-      </c>
     </row>
-    <row r="3" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
-      <c r="B3" s="52"/>
-      <c r="C3" s="53" t="s">
+    <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="93"/>
+      <c r="B3" s="91"/>
+      <c r="C3" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D3" s="54">
-        <v>0</v>
-      </c>
-      <c r="E3" s="54">
-        <v>0</v>
-      </c>
-      <c r="F3" s="54">
-        <v>0</v>
-      </c>
-      <c r="G3" s="54">
-        <v>0</v>
-      </c>
-      <c r="H3" s="54">
-        <v>0</v>
-      </c>
-      <c r="I3" s="54">
-        <v>0</v>
-      </c>
-      <c r="J3" s="54">
-        <v>0</v>
-      </c>
-      <c r="K3" s="54">
-        <v>0</v>
-      </c>
-      <c r="L3" s="54">
-        <v>0</v>
-      </c>
-      <c r="M3" s="54">
-        <v>0</v>
-      </c>
-      <c r="N3" s="54">
-        <v>0</v>
-      </c>
-      <c r="O3" s="54">
-        <v>0</v>
-      </c>
-      <c r="P3" s="58">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="63"/>
-      <c r="R3" s="53"/>
-      <c r="S3" s="53"/>
-      <c r="T3" s="55"/>
+      <c r="D3" s="23">
+        <v>0.87</v>
+      </c>
+      <c r="E3" s="23">
+        <v>1</v>
+      </c>
+      <c r="F3" s="23">
+        <v>1</v>
+      </c>
+      <c r="G3" s="23">
+        <v>1</v>
+      </c>
+      <c r="H3" s="23">
+        <v>1</v>
+      </c>
+      <c r="I3" s="23">
+        <v>0.75</v>
+      </c>
+      <c r="J3" s="23">
+        <v>1</v>
+      </c>
+      <c r="K3" s="23">
+        <v>1</v>
+      </c>
+      <c r="L3" s="23">
+        <v>1</v>
+      </c>
+      <c r="M3" s="23">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="N3" s="23">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="O3" s="23">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="P3" s="26">
+        <v>0.5</v>
+      </c>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Anteproyectos: 3 proyectos PAEB y hojas AVAN con varias tablas
- Datos: nuevo Excel (PAEB Agua Prieta, Zimapán-Alternativa B y Benito
  Juárez) y KML con sus ubicaciones.
- Lector: "Proyecto de Acumulación de Energía por Bombeo" usa las hojas
  _PAEB. Una hoja AVAN puede tener varias tablas (una por proyecto, cada
  una con su fila "No."): cada proyecto toma los ponderados y notas de su
  tabla. Un número repetido en los encabezados (1.10 que Excel cambia a
  1.1) es error, con la indicación de escribir '1.10.
- Sin foto, los PAEB muestran el ícono hidráulico.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01APiq7bAy76yveceNZKtsYf
</commit_message>
<xml_diff>
--- a/cartera-anteproyectos/data/datos_anteproyectos.xlsx
+++ b/cartera-anteproyectos/data/datos_anteproyectos.xlsx
@@ -1,33 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CN594\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F2C11E4-E5DB-49E8-BCB4-279A5BB3DC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A888A5-C762-40AD-B5C6-798BFD97F084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="839" xr2:uid="{F77216BA-A0B8-4B6C-9AC8-5CF7CF39AEC5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="925" activeTab="3" xr2:uid="{F77216BA-A0B8-4B6C-9AC8-5CF7CF39AEC5}"/>
   </bookViews>
   <sheets>
     <sheet name="PRES" sheetId="1" r:id="rId1"/>
     <sheet name="DESC" sheetId="3" r:id="rId2"/>
     <sheet name="RTA" sheetId="5" r:id="rId3"/>
-    <sheet name="FICHA_FOTOV" sheetId="2" r:id="rId4"/>
-    <sheet name="AVAN_FOTOV" sheetId="4" r:id="rId5"/>
-    <sheet name="FICHA_TERSOL" sheetId="6" r:id="rId6"/>
-    <sheet name="AVAN_TERSOL" sheetId="7" r:id="rId7"/>
-    <sheet name="FICHA_EO" sheetId="8" r:id="rId8"/>
-    <sheet name="AVAN_EO" sheetId="9" r:id="rId9"/>
-    <sheet name="FICHA_EQUIHIDRO" sheetId="10" r:id="rId10"/>
-    <sheet name="AVAN_EQUIHIDRO" sheetId="11" r:id="rId11"/>
-    <sheet name="FICHA_HIDRO" sheetId="12" r:id="rId12"/>
-    <sheet name="AVAN_HIDRO" sheetId="13" r:id="rId13"/>
+    <sheet name="FICHA_PAEB" sheetId="14" r:id="rId4"/>
+    <sheet name="AVAN_PAEB" sheetId="15" r:id="rId5"/>
+    <sheet name="FICHA_FOTOV" sheetId="2" r:id="rId6"/>
+    <sheet name="AVAN_FOTOV" sheetId="4" r:id="rId7"/>
+    <sheet name="FICHA_TERSOL" sheetId="6" r:id="rId8"/>
+    <sheet name="AVAN_TERSOL" sheetId="7" r:id="rId9"/>
+    <sheet name="FICHA_EO" sheetId="8" r:id="rId10"/>
+    <sheet name="AVAN_EO" sheetId="9" r:id="rId11"/>
+    <sheet name="FICHA_EQUIHIDRO" sheetId="10" r:id="rId12"/>
+    <sheet name="AVAN_EQUIHIDRO" sheetId="11" r:id="rId13"/>
+    <sheet name="FICHA_HIDRO" sheetId="12" r:id="rId14"/>
+    <sheet name="AVAN_HIDRO" sheetId="13" r:id="rId15"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">FICHA_PAEB!$A$1:$N$1</definedName>
+  </definedNames>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -51,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="267">
   <si>
     <t>PFV Isla Cayacal (Petacalco)</t>
   </si>
@@ -502,6 +507,408 @@
   </si>
   <si>
     <t>NOTA (1.3)</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>PAEB Zimapán-Alternativa B</t>
+  </si>
+  <si>
+    <t>PAEB Agua Prieta</t>
+  </si>
+  <si>
+    <t>PAEB Benito Juárez</t>
+  </si>
+  <si>
+    <t>Gran Visión</t>
+  </si>
+  <si>
+    <t>Proyecto de Acumulación de Energía por Bombeo</t>
+  </si>
+  <si>
+    <t>Zapopan, Jalisco</t>
+  </si>
+  <si>
+    <t>Tecozautla, Hidalgo</t>
+  </si>
+  <si>
+    <t>Santa María Jalapa del Marqués, Oaxaca</t>
+  </si>
+  <si>
+    <t>data/IMAGENES/AGUA_PRIETA.jpg</t>
+  </si>
+  <si>
+    <t>data/IMAGENES/ZIMAPAN.jpg</t>
+  </si>
+  <si>
+    <t>data/IMAGENES/OAXACA.jpg</t>
+  </si>
+  <si>
+    <t>El Proyecto de Acumulación de Energía por Bombeo (PAEB) Agua Prieta, plantea aprovechar parte de la infraestructura de la CH Agua Prieta, principalmente el actual tanque sedimentador y regulador, como tanque superior para el PAEB, integrando una tubería que conducirá a una casa de máquinas en caverna equipada con 2 equipos turbogeneradores con turbinas Francis reversibles y una estructura contenedora sobre el río Santiago como tanque inferior, con el objetivo de bombear hacia el tanque superior y generar hacia el tanque inferior. 
+El diseño del PAEB considerará las condiciones de operación de la CH Agua Prieta y se integrará de las obras tales como:
+1. Tanque superior
+2. Túnel y tubería de conducción
+3. Casa de máquinas
+4. Tanque inferior
+5. Subestación elevadora
+6. Interconexión</t>
+  </si>
+  <si>
+    <t>El Proyecto de Acumulación de Energía por Bombeo (PAEB) Zimapán, aprovechará el embalse de la presa Zimapán de la CH Fernando Hiriart Balderrama y se busca la mejor opción para el diseño del vaso superior, mediante el estudio de viabilidad técnica, socioambiental, jurídica del predio, arqueológica y financiera de ocho alternativas en los municipios de Querétaro e Hidalgo.
+La PAEB Zimapán está integrado por un tanque elevado excavado (1.86 Mm3), tubería a presión (Diam 4.6 m), casa de máquinas tipo galería (2U reversibles) tipo Francis, un tanque inferior-Presa Zimapán, subestación elevadora, línea al punto de interconexión y subestación de maniobras.
+El diseño del PAEB considerará las condiciones de operación de la CH Zimapán y se integrará de las obras tales como:
+1. Tanque superior
+2. Túnel y tubería de conducción
+3. Casa de máquinas
+4. Tanque inferior (embalse Zimapán)
+5. Subestación elevadora
+6. Línea de interconexión-230 kV
+6. Interconexión (SE-Maniobras)</t>
+  </si>
+  <si>
+    <t>Comprende la elaboración de un esquema de aprovechamiento de rebombeo utilizando como embalse inferior el correspondiente a la presa Benito Juárez, sin afectar la política de operación actual de ésta y sus compromisos hídricos. Eliminando la necesidad de construir un embalse inferior el objetivo es localizar un sitio factible para el emplazamiento del tanque superior con la capacidad de suministrar la potencia y energía requeridas en la red.
+A continuación, se listan las seis obras principales del proyecto:
+1. Tanque superior
+2. Conducción
+3. Casa de máquinas
+4. Desfogue
+5. Subestación elevadora
+6. Interconexión</t>
+  </si>
+  <si>
+    <t>2 Circuitos</t>
+  </si>
+  <si>
+    <t>Minimización del trazado para reducir pérdidas técnicas y costos de inversión en conductor y contar con capacidad en el NODO</t>
+  </si>
+  <si>
+    <t>Alejamiento de zonas de alta densidad poblacional</t>
+  </si>
+  <si>
+    <t>230/34 kV, Transformador ppal.</t>
+  </si>
+  <si>
+    <t>2 Bahías</t>
+  </si>
+  <si>
+    <t>Subestación Guadalajara Norte</t>
+  </si>
+  <si>
+    <t>Conexión en el nodo 03GUN-230 de la SE Guadalajara Norte del sistema de transmisión nacional/regional.</t>
+  </si>
+  <si>
+    <t>Alejamiento de zonas de alta densidad poblacional. No se encuentran dentro de alguna área de conservación (i. e., ANP's, AICAS, Sitios RAMSAR).</t>
+  </si>
+  <si>
+    <t>47 Unid.</t>
+  </si>
+  <si>
+    <t>Subestación Dañu</t>
+  </si>
+  <si>
+    <t>Conexión en el nodo del circuito 93060, LT-Zimapán PH-DAÑU, Occidente del sistema de transmisión nacional/regional.</t>
+  </si>
+  <si>
+    <t>Por definir</t>
+  </si>
+  <si>
+    <t>Transformador ppal.</t>
+  </si>
+  <si>
+    <t>Subestación Ixtepec Potencia</t>
+  </si>
+  <si>
+    <t>Interconexión en el nodo 02IPO - 230 de la SE Ixtepec Potencia del sistema de transmisión nacional/regional</t>
+  </si>
+  <si>
+    <t>Factor de planta [%]</t>
+  </si>
+  <si>
+    <t>Gasto de Diseño [m3/s]</t>
+  </si>
+  <si>
+    <t>Volumen útil [hm3]</t>
+  </si>
+  <si>
+    <t>Nodo de interconexión</t>
+  </si>
+  <si>
+    <t>CAPEX (MUSD)</t>
+  </si>
+  <si>
+    <t>OPEX (MUSD/Año)</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>828</t>
+  </si>
+  <si>
+    <t>S.E. Guadalajara Norte</t>
+  </si>
+  <si>
+    <t>240</t>
+  </si>
+  <si>
+    <t>380</t>
+  </si>
+  <si>
+    <t>17.9</t>
+  </si>
+  <si>
+    <t>Francis Reversibles</t>
+  </si>
+  <si>
+    <t>0.77</t>
+  </si>
+  <si>
+    <t>51.7</t>
+  </si>
+  <si>
+    <t>513</t>
+  </si>
+  <si>
+    <t>0.8</t>
+  </si>
+  <si>
+    <t>197</t>
+  </si>
+  <si>
+    <t>431.71</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>0.0048</t>
+  </si>
+  <si>
+    <t>86.28</t>
+  </si>
+  <si>
+    <t>240.26</t>
+  </si>
+  <si>
+    <t>2.081</t>
+  </si>
+  <si>
+    <t>S.E. Dañú</t>
+  </si>
+  <si>
+    <t>702.5</t>
+  </si>
+  <si>
+    <t>4.75</t>
+  </si>
+  <si>
+    <t>Sin dato</t>
+  </si>
+  <si>
+    <t>S.E. Ixtepec potencia</t>
+  </si>
+  <si>
+    <t>2.7</t>
+  </si>
+  <si>
+    <t>543</t>
+  </si>
+  <si>
+    <t>189.51</t>
+  </si>
+  <si>
+    <t>16.7</t>
+  </si>
+  <si>
+    <t>1314</t>
+  </si>
+  <si>
+    <t>900</t>
+  </si>
+  <si>
+    <t>1.1 Análisis de la disponibilidad del recurso hídrico.</t>
+  </si>
+  <si>
+    <t>1.2 Certidumbre de los terrenos a ocupar.</t>
+  </si>
+  <si>
+    <t>1.3 Diagnóstico social preliminar.</t>
+  </si>
+  <si>
+    <t>1.4 Diagnóstico ambiental preliminar.</t>
+  </si>
+  <si>
+    <t>1.5 Diagnóstico arqueológico preliminar.</t>
+  </si>
+  <si>
+    <t>1.6 Análisis FODA.</t>
+  </si>
+  <si>
+    <t>2.2 Levantamiento topográfico LiDAR con Dron, 7 de agosto</t>
+  </si>
+  <si>
+    <t>2.3 Análisis de la operación de la CH Agua Prieta y estudio hidrológico.</t>
+  </si>
+  <si>
+    <t>2.4 Planteamiento de obras principales</t>
+  </si>
+  <si>
+    <t>2.5 Análisis hidroenergético.</t>
+  </si>
+  <si>
+    <t>2.6 Obras complementarias requeridas.</t>
+  </si>
+  <si>
+    <t>2.7 Estimación preliminar de CAPEX , OPEX y programa de obra.</t>
+  </si>
+  <si>
+    <t>1. Certidumbre Social, Ambiental, Tenencia de la tierra e Hídrica</t>
+  </si>
+  <si>
+    <t>•	Levantamiento topográfico en campo, se concluye el informe el 14 de agosto.
+•	El 09 de octubre se recibió información técnica de la CH Agua Prieta, ésta se utilizará para el planteamiento del proyecto de rebombeo.
+•	Se realiza análisis hidrológico e hidroenergético, así como planteamientos de aprovechamiento hidroeléctrico como PAEB y como bombeo del río Santiago al tanque superior actual para incrementar FP de la CH Agua Prieta.
+•	Se mapean terrenos externos a los de CFE y se ha identificado Núcleos Agrarios.
+•	Se planea 2da visita técnica en noviembre de 2026.
+•	Se continúa con gestión de la Clave de Registro Única para desarrollar los Estudios de Preinversión a partir de marzo de 2027.</t>
+  </si>
+  <si>
+    <t>Se requiere reunión con CONAGUA para verificar Concesión de agua</t>
+  </si>
+  <si>
+    <t>Pendiente segunda visita técnica</t>
+  </si>
+  <si>
+    <t>NOTA (2.1)</t>
+  </si>
+  <si>
+    <t>NOTA (2.3)</t>
+  </si>
+  <si>
+    <t>Se realizan análisis con información disponible</t>
+  </si>
+  <si>
+    <t>1 Planteamiento de sitios aprovechables</t>
+  </si>
+  <si>
+    <t>1.1  Disponibilidad y factibilidad del uso del recurso hídrico</t>
+  </si>
+  <si>
+    <t>1.2  Topografía</t>
+  </si>
+  <si>
+    <t>1.3  Análisis de riesgos y áreas restringidas</t>
+  </si>
+  <si>
+    <t>1.4  Propuesta de interconexión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.5   Diagnóstico ambiental </t>
+  </si>
+  <si>
+    <t>1.6   Diagnóstico Social</t>
+  </si>
+  <si>
+    <t>1.7   Diagnóstico Arqueológico</t>
+  </si>
+  <si>
+    <t>1.8   Diagnóstico de la Certidumbre jurídica del predio</t>
+  </si>
+  <si>
+    <t>2.1  Evaluación de la viabilidad técnica de alternativas</t>
+  </si>
+  <si>
+    <t>2.2  Opción definitiva</t>
+  </si>
+  <si>
+    <t>2.3  Presupuesto</t>
+  </si>
+  <si>
+    <t>2.4  Gestión del presupuesto para preinversión</t>
+  </si>
+  <si>
+    <t>2.5  Informe</t>
+  </si>
+  <si>
+    <t>2. Análisis, priorización y selección de sitios</t>
+  </si>
+  <si>
+    <t>•	Con base en la consulta realizada a la Subestación 1 Querétaro, se planteó propuesta de interconexión, conexión a la LT de 230 kV que va de Zimapán a Tula.
+•	Se realiza un análisis comparativo de alternativas para la evaluación técnica, ambiental, social y arqueológica para determinar de opción más viable.
+•	Se concertará cita a finales de noviembre con la zona de transmisión Centro/Poniente de la región de Tula, encargada de operar y mantener las redes de alta tensión. Para evaluar la propuesta del punto de interconexión que corresponde a la Subestación Dañu.
+•	Se coordina la visita con el personal de la central hidroeléctrica (noviembre 2026).</t>
+  </si>
+  <si>
+    <t>Se confirmó la disponibilidad del agua</t>
+  </si>
+  <si>
+    <t>Se complementará el análisis con identificación en campo</t>
+  </si>
+  <si>
+    <t>Solo sitio 5, 6- Ejidos (registro RAN)</t>
+  </si>
+  <si>
+    <t>Se seleccionarán 2 opciones para estudio en campo.</t>
+  </si>
+  <si>
+    <t>1.1   Análisis de la disponibilidad y factibilidad del uso del recurso hídrico</t>
+  </si>
+  <si>
+    <t>1.2   Topografía</t>
+  </si>
+  <si>
+    <t>1.3   Análisis de riesgos y áreas restringidas</t>
+  </si>
+  <si>
+    <t>1.4  Diagnóstico de la Certidumbre jurídica del predio</t>
+  </si>
+  <si>
+    <t>1.5   Análisis de demanda y generación de energía eléctrica</t>
+  </si>
+  <si>
+    <t>1.6   Análisis de la red eléctrica</t>
+  </si>
+  <si>
+    <t>1.7   Propuesta de interconexión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.8   Diagnóstico ambiental </t>
+  </si>
+  <si>
+    <t>1.9   Diagnóstico Social</t>
+  </si>
+  <si>
+    <t>2.1   Evaluación de la viabilidad técnica de alternativas</t>
+  </si>
+  <si>
+    <t>2.2 Opción definitiva</t>
+  </si>
+  <si>
+    <t>2.3   Presupuesto</t>
+  </si>
+  <si>
+    <t>2.4   Gestión del presupuesto para preinversión</t>
+  </si>
+  <si>
+    <t>1. Planteamiento de sitios aprovechables</t>
+  </si>
+  <si>
+    <t>2. Análisis, priorización y selección de sitios.</t>
+  </si>
+  <si>
+    <t>•	Las actividades 1 y 2 se requiere información actualizada, se hará la gestión social para visita en campo que permita desarrollar los trabajo para topografía LiDAR y batimetría.
+•	Se propone una visita multidisciplinaria al sitio, condicionada a la realización de las gestiones sociales correspondientes. Paralelamente, se elabora la cartografía social y los guiones de entrevista para las actividades de investigación en campo con autoridades municipales y funcionarios del Distrito de Riego 19.
+•	Las actividades 4 y 5 se gestionará información acerca del nodo de interconexión.
+•	El diagnostico ambiental se pauso TEMPORALMENTE.
+•	En materia social: Avances en un 60% (Contextualización), planificación de reunión de trabajo con personal del Organismo de Cuenca Pacífico Sur. 
+•	Visita multidisciplinaria al sitio, condicionada a la realización de las gestiones sociales correspondientes. Paralelamente, se elabora la cartografía social y los guiones de entrevista para las actividades de investigación en campo con autoridades municipales y funcionarios del Distrito de Riego 19.</t>
+  </si>
+  <si>
+    <t>1.10  Diagnóstico Arqueológico</t>
   </si>
 </sst>
 </file>
@@ -1232,7 +1639,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1322,6 +1729,131 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="42" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1332,75 +1864,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1410,6 +1873,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFC72965"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1738,14 +2206,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7582F8E4-5871-4CE4-85C7-5CB4D3DD57AE}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="26.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="31" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.42578125" style="1"/>
     <col min="8" max="8" width="11.42578125" style="1" customWidth="1"/>
@@ -1812,18 +2280,102 @@
         <v>98</v>
       </c>
     </row>
+    <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="33" t="s">
+        <v>145</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>148</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>151</v>
+      </c>
+      <c r="E4" s="34" t="s">
+        <v>152</v>
+      </c>
+      <c r="F4" s="38" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>151</v>
+      </c>
+      <c r="E5" s="34" t="s">
+        <v>153</v>
+      </c>
+      <c r="F5" s="38" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>151</v>
+      </c>
+      <c r="E6" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="F6" s="38" t="s">
+        <v>157</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEB907A7-035C-4DD7-877C-3D230C7BC692}">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C60ADB6-D9A9-438B-98FC-D53C5C09C361}">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11391311-F088-476E-AA2B-249B6F9FAC1E}">
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="23" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.42578125" bestFit="1" customWidth="1"/>
@@ -1932,13 +2484,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{454BA043-9B01-4C3D-9384-998F797746DE}">
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:V3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -2016,10 +2568,10 @@
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="116" t="s">
         <v>94</v>
       </c>
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="118" t="s">
         <v>95</v>
       </c>
       <c r="C2" s="4" t="s">
@@ -2084,8 +2636,8 @@
       </c>
     </row>
     <row r="3" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="68"/>
-      <c r="B3" s="70"/>
+      <c r="A3" s="117"/>
+      <c r="B3" s="119"/>
       <c r="C3" s="7" t="s">
         <v>39</v>
       </c>
@@ -2150,25 +2702,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D74E2DAE-8635-40A7-B7FB-1F37778E2B23}">
   <sheetPr>
     <tabColor theme="8" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2F8F003-E05E-4325-8F16-62CE7B570DCC}">
   <sheetPr>
     <tabColor theme="8" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2176,8 +2728,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45D77318-4E74-4035-A05D-AC6B6DDDAC7C}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
@@ -2217,6 +2769,39 @@
         <v>99</v>
       </c>
     </row>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="33" t="s">
+        <v>145</v>
+      </c>
+      <c r="B4" s="34" t="s">
+        <v>148</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="34" t="s">
+        <v>160</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2224,8 +2809,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37E307FA-5186-457C-8CE8-B07656929254}">
-  <dimension ref="A1:Q11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Q23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
@@ -2243,54 +2828,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="86" t="s">
+      <c r="A1" s="100" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="87"/>
-      <c r="C1" s="87"/>
-      <c r="D1" s="87"/>
-      <c r="E1" s="87"/>
-      <c r="F1" s="87"/>
-      <c r="G1" s="87"/>
-      <c r="H1" s="87"/>
-      <c r="I1" s="87"/>
-      <c r="J1" s="87"/>
-      <c r="K1" s="87"/>
-      <c r="L1" s="87"/>
-      <c r="M1" s="87"/>
-      <c r="N1" s="87"/>
-      <c r="O1" s="87"/>
-      <c r="P1" s="87"/>
-      <c r="Q1" s="88"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="101"/>
+      <c r="G1" s="101"/>
+      <c r="H1" s="101"/>
+      <c r="I1" s="101"/>
+      <c r="J1" s="101"/>
+      <c r="K1" s="101"/>
+      <c r="L1" s="101"/>
+      <c r="M1" s="101"/>
+      <c r="N1" s="101"/>
+      <c r="O1" s="101"/>
+      <c r="P1" s="101"/>
+      <c r="Q1" s="102"/>
     </row>
     <row r="2" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="77" t="s">
+      <c r="A2" s="91" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="78"/>
-      <c r="C2" s="77" t="s">
+      <c r="B2" s="92"/>
+      <c r="C2" s="91" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="77" t="s">
+      <c r="D2" s="99"/>
+      <c r="E2" s="99"/>
+      <c r="F2" s="99"/>
+      <c r="G2" s="99"/>
+      <c r="H2" s="92"/>
+      <c r="I2" s="91" t="s">
         <v>61</v>
       </c>
-      <c r="J2" s="85"/>
-      <c r="K2" s="78"/>
-      <c r="L2" s="77" t="s">
+      <c r="J2" s="99"/>
+      <c r="K2" s="92"/>
+      <c r="L2" s="91" t="s">
         <v>89</v>
       </c>
-      <c r="M2" s="85"/>
-      <c r="N2" s="89"/>
-      <c r="O2" s="77" t="s">
+      <c r="M2" s="99"/>
+      <c r="N2" s="103"/>
+      <c r="O2" s="91" t="s">
         <v>90</v>
       </c>
-      <c r="P2" s="85"/>
-      <c r="Q2" s="78"/>
+      <c r="P2" s="99"/>
+      <c r="Q2" s="92"/>
     </row>
     <row r="3" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="65" t="s">
@@ -2346,10 +2931,10 @@
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="79">
+      <c r="A4" s="93">
         <v>1</v>
       </c>
-      <c r="B4" s="82" t="s">
+      <c r="B4" s="96" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="55">
@@ -2399,8 +2984,8 @@
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="80"/>
-      <c r="B5" s="83"/>
+      <c r="A5" s="94"/>
+      <c r="B5" s="97"/>
       <c r="H5" s="12"/>
       <c r="I5" s="11"/>
       <c r="K5" s="12"/>
@@ -2417,8 +3002,8 @@
       <c r="Q5" s="12"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="80"/>
-      <c r="B6" s="83"/>
+      <c r="A6" s="94"/>
+      <c r="B6" s="97"/>
       <c r="H6" s="12"/>
       <c r="I6" s="11"/>
       <c r="K6" s="12"/>
@@ -2435,8 +3020,8 @@
       <c r="Q6" s="12"/>
     </row>
     <row r="7" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="81"/>
-      <c r="B7" s="84"/>
+      <c r="A7" s="95"/>
+      <c r="B7" s="98"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
@@ -2460,10 +3045,10 @@
       <c r="Q7" s="14"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="74" t="s">
+      <c r="A8" s="88" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="71" t="s">
+      <c r="B8" s="85" t="s">
         <v>95</v>
       </c>
       <c r="C8" s="50">
@@ -2513,8 +3098,8 @@
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="75"/>
-      <c r="B9" s="72"/>
+      <c r="A9" s="89"/>
+      <c r="B9" s="86"/>
       <c r="H9" s="12"/>
       <c r="I9" s="11"/>
       <c r="K9" s="12"/>
@@ -2531,8 +3116,8 @@
       <c r="Q9" s="12"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="75"/>
-      <c r="B10" s="72"/>
+      <c r="A10" s="89"/>
+      <c r="B10" s="86"/>
       <c r="H10" s="12"/>
       <c r="I10" s="11"/>
       <c r="K10" s="12"/>
@@ -2549,8 +3134,8 @@
       <c r="Q10" s="12"/>
     </row>
     <row r="11" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="76"/>
-      <c r="B11" s="73"/>
+      <c r="A11" s="90"/>
+      <c r="B11" s="87"/>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
@@ -2573,8 +3158,356 @@
       <c r="P11" s="7"/>
       <c r="Q11" s="14"/>
     </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" s="104" t="s">
+        <v>145</v>
+      </c>
+      <c r="B12" s="107" t="s">
+        <v>148</v>
+      </c>
+      <c r="C12" s="50">
+        <v>230</v>
+      </c>
+      <c r="D12" s="51">
+        <v>240</v>
+      </c>
+      <c r="E12" s="51" t="s">
+        <v>57</v>
+      </c>
+      <c r="F12" s="51">
+        <v>3.3</v>
+      </c>
+      <c r="G12" s="51" t="s">
+        <v>161</v>
+      </c>
+      <c r="H12" s="52" t="s">
+        <v>60</v>
+      </c>
+      <c r="I12" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="J12" s="48" t="s">
+        <v>163</v>
+      </c>
+      <c r="K12" s="49" t="s">
+        <v>67</v>
+      </c>
+      <c r="L12" s="53" t="s">
+        <v>68</v>
+      </c>
+      <c r="M12" s="45" t="s">
+        <v>101</v>
+      </c>
+      <c r="N12" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="O12" s="47" t="s">
+        <v>166</v>
+      </c>
+      <c r="P12" s="48" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q12" s="49" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" s="105"/>
+      <c r="B13" s="108"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="11"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="N13" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="O13" s="11"/>
+      <c r="Q13" s="12"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" s="105"/>
+      <c r="B14" s="108"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="11"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="N14" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="O14" s="11"/>
+      <c r="Q14" s="12"/>
+    </row>
+    <row r="15" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="106"/>
+      <c r="B15" s="109"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="14"/>
+      <c r="L15" s="54" t="s">
+        <v>71</v>
+      </c>
+      <c r="M15" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="N15" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="O15" s="13"/>
+      <c r="P15" s="7"/>
+      <c r="Q15" s="14"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" s="104" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" s="107" t="s">
+        <v>147</v>
+      </c>
+      <c r="C16" s="50">
+        <v>230</v>
+      </c>
+      <c r="D16" s="51">
+        <v>197</v>
+      </c>
+      <c r="E16" s="51" t="s">
+        <v>57</v>
+      </c>
+      <c r="F16" s="51">
+        <v>6.2</v>
+      </c>
+      <c r="G16" s="51" t="s">
+        <v>161</v>
+      </c>
+      <c r="H16" s="52" t="s">
+        <v>60</v>
+      </c>
+      <c r="I16" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="J16" s="48" t="s">
+        <v>168</v>
+      </c>
+      <c r="K16" s="49" t="s">
+        <v>67</v>
+      </c>
+      <c r="L16" s="53" t="s">
+        <v>68</v>
+      </c>
+      <c r="M16" s="45" t="s">
+        <v>101</v>
+      </c>
+      <c r="N16" s="46" t="s">
+        <v>169</v>
+      </c>
+      <c r="O16" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="P16" s="48" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q16" s="49" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A17" s="105"/>
+      <c r="B17" s="108"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="11"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="N17" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="O17" s="11"/>
+      <c r="Q17" s="12"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A18" s="105"/>
+      <c r="B18" s="108"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="11"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="N18" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="O18" s="11"/>
+      <c r="Q18" s="12"/>
+    </row>
+    <row r="19" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="106"/>
+      <c r="B19" s="109"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="54" t="s">
+        <v>71</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="N19" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="O19" s="13"/>
+      <c r="P19" s="7"/>
+      <c r="Q19" s="14"/>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A20" s="104" t="s">
+        <v>146</v>
+      </c>
+      <c r="B20" s="107" t="s">
+        <v>149</v>
+      </c>
+      <c r="C20" s="50">
+        <v>400</v>
+      </c>
+      <c r="D20" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="E20" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="F20" s="51">
+        <v>56</v>
+      </c>
+      <c r="G20" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="H20" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="I20" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="J20" s="48" t="s">
+        <v>163</v>
+      </c>
+      <c r="K20" s="49" t="s">
+        <v>67</v>
+      </c>
+      <c r="L20" s="53" t="s">
+        <v>68</v>
+      </c>
+      <c r="M20" s="45" t="s">
+        <v>101</v>
+      </c>
+      <c r="N20" s="46" t="s">
+        <v>172</v>
+      </c>
+      <c r="O20" s="47" t="s">
+        <v>174</v>
+      </c>
+      <c r="P20" s="48" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q20" s="49" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A21" s="105"/>
+      <c r="B21" s="108"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="11"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="N21" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="O21" s="11"/>
+      <c r="Q21" s="12"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A22" s="105"/>
+      <c r="B22" s="108"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="11"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="N22" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="O22" s="11"/>
+      <c r="Q22" s="12"/>
+    </row>
+    <row r="23" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="106"/>
+      <c r="B23" s="109"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="14"/>
+      <c r="L23" s="54" t="s">
+        <v>71</v>
+      </c>
+      <c r="M23" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="N23" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="O23" s="13"/>
+      <c r="P23" s="7"/>
+      <c r="Q23" s="14"/>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="16">
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="B12:B15"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="B16:B19"/>
     <mergeCell ref="O2:Q2"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="C2:H2"/>
@@ -2591,12 +3524,886 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D05FE715-3CBD-460A-B083-689D25D850F4}">
+  <sheetPr>
+    <tabColor rgb="FFC72965"/>
+  </sheetPr>
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="69" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="70" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="70" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1" s="70" t="s">
+        <v>109</v>
+      </c>
+      <c r="E1" s="70" t="s">
+        <v>176</v>
+      </c>
+      <c r="F1" s="70" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="H1" s="70" t="s">
+        <v>115</v>
+      </c>
+      <c r="I1" s="70" t="s">
+        <v>177</v>
+      </c>
+      <c r="J1" s="70" t="s">
+        <v>119</v>
+      </c>
+      <c r="K1" s="70" t="s">
+        <v>178</v>
+      </c>
+      <c r="L1" s="70" t="s">
+        <v>179</v>
+      </c>
+      <c r="M1" s="70" t="s">
+        <v>180</v>
+      </c>
+      <c r="N1" s="70" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="67" t="s">
+        <v>145</v>
+      </c>
+      <c r="B2" s="68" t="s">
+        <v>148</v>
+      </c>
+      <c r="C2" s="68" t="s">
+        <v>185</v>
+      </c>
+      <c r="D2" s="68" t="s">
+        <v>186</v>
+      </c>
+      <c r="E2" s="68" t="s">
+        <v>187</v>
+      </c>
+      <c r="F2" s="68" t="s">
+        <v>94</v>
+      </c>
+      <c r="G2" s="68" t="s">
+        <v>188</v>
+      </c>
+      <c r="H2" s="68" t="s">
+        <v>189</v>
+      </c>
+      <c r="I2" s="68" t="s">
+        <v>190</v>
+      </c>
+      <c r="J2" s="68" t="s">
+        <v>191</v>
+      </c>
+      <c r="K2" s="68" t="s">
+        <v>192</v>
+      </c>
+      <c r="L2" s="68" t="s">
+        <v>184</v>
+      </c>
+      <c r="M2" s="68" t="s">
+        <v>183</v>
+      </c>
+      <c r="N2" s="68" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" s="38" t="s">
+        <v>147</v>
+      </c>
+      <c r="C3" s="38" t="s">
+        <v>193</v>
+      </c>
+      <c r="D3" s="38" t="s">
+        <v>194</v>
+      </c>
+      <c r="E3" s="38" t="s">
+        <v>195</v>
+      </c>
+      <c r="F3" s="38" t="s">
+        <v>94</v>
+      </c>
+      <c r="G3" s="68" t="s">
+        <v>188</v>
+      </c>
+      <c r="H3" s="38" t="s">
+        <v>196</v>
+      </c>
+      <c r="I3" s="38" t="s">
+        <v>197</v>
+      </c>
+      <c r="J3" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="K3" s="38" t="s">
+        <v>199</v>
+      </c>
+      <c r="L3" s="38" t="s">
+        <v>200</v>
+      </c>
+      <c r="M3" s="38" t="s">
+        <v>201</v>
+      </c>
+      <c r="N3" s="38" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="C4" s="38" t="s">
+        <v>210</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="E4" s="38" t="s">
+        <v>208</v>
+      </c>
+      <c r="F4" s="38" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="68" t="s">
+        <v>188</v>
+      </c>
+      <c r="H4" s="38" t="s">
+        <v>116</v>
+      </c>
+      <c r="I4" s="38" t="s">
+        <v>207</v>
+      </c>
+      <c r="J4" s="38" t="s">
+        <v>206</v>
+      </c>
+      <c r="K4" s="38" t="s">
+        <v>205</v>
+      </c>
+      <c r="L4" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="M4" s="38" t="s">
+        <v>203</v>
+      </c>
+      <c r="N4" s="38" t="s">
+        <v>203</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N1" xr:uid="{D05FE715-3CBD-460A-B083-689D25D850F4}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77E019FD-B91C-4FC3-9118-94588F3A8D19}">
+  <sheetPr>
+    <tabColor rgb="FFC72965"/>
+  </sheetPr>
+  <dimension ref="A1:X11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="21" max="21" width="11.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="80" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="81" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="81" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="81" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="81" t="s">
+        <v>223</v>
+      </c>
+      <c r="F1" s="81" t="s">
+        <v>211</v>
+      </c>
+      <c r="G1" s="81" t="s">
+        <v>212</v>
+      </c>
+      <c r="H1" s="81" t="s">
+        <v>213</v>
+      </c>
+      <c r="I1" s="81" t="s">
+        <v>214</v>
+      </c>
+      <c r="J1" s="81" t="s">
+        <v>215</v>
+      </c>
+      <c r="K1" s="81" t="s">
+        <v>216</v>
+      </c>
+      <c r="L1" s="81" t="s">
+        <v>34</v>
+      </c>
+      <c r="M1" s="81" t="s">
+        <v>134</v>
+      </c>
+      <c r="N1" s="81" t="s">
+        <v>217</v>
+      </c>
+      <c r="O1" s="81" t="s">
+        <v>218</v>
+      </c>
+      <c r="P1" s="81" t="s">
+        <v>219</v>
+      </c>
+      <c r="Q1" s="81" t="s">
+        <v>220</v>
+      </c>
+      <c r="R1" s="81" t="s">
+        <v>221</v>
+      </c>
+      <c r="S1" s="82" t="s">
+        <v>222</v>
+      </c>
+      <c r="T1" s="76" t="s">
+        <v>49</v>
+      </c>
+      <c r="U1" s="73" t="s">
+        <v>142</v>
+      </c>
+      <c r="V1" s="73" t="s">
+        <v>227</v>
+      </c>
+      <c r="W1" s="71" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A2" s="89" t="s">
+        <v>145</v>
+      </c>
+      <c r="B2" s="110" t="s">
+        <v>148</v>
+      </c>
+      <c r="C2" s="75" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="72">
+        <v>0.42</v>
+      </c>
+      <c r="E2" s="72">
+        <v>0.5</v>
+      </c>
+      <c r="F2" s="72">
+        <v>0.5</v>
+      </c>
+      <c r="G2" s="72">
+        <v>0.7</v>
+      </c>
+      <c r="H2" s="72">
+        <v>0.7</v>
+      </c>
+      <c r="I2" s="72">
+        <v>0.5</v>
+      </c>
+      <c r="J2" s="72">
+        <v>0.6</v>
+      </c>
+      <c r="K2" s="72">
+        <v>0</v>
+      </c>
+      <c r="L2" s="72">
+        <v>0.33</v>
+      </c>
+      <c r="M2" s="72">
+        <v>0.5</v>
+      </c>
+      <c r="N2" s="72">
+        <v>1</v>
+      </c>
+      <c r="O2" s="72">
+        <v>0.3</v>
+      </c>
+      <c r="P2" s="72">
+        <v>0.35</v>
+      </c>
+      <c r="Q2" s="72">
+        <v>0.1</v>
+      </c>
+      <c r="R2" s="72">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="S2" s="77">
+        <v>0</v>
+      </c>
+      <c r="T2" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="U2" t="s">
+        <v>225</v>
+      </c>
+      <c r="V2" t="s">
+        <v>226</v>
+      </c>
+      <c r="W2" s="12" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="90"/>
+      <c r="B3" s="111"/>
+      <c r="C3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="78">
+        <v>0.61</v>
+      </c>
+      <c r="E3" s="78">
+        <v>0.6</v>
+      </c>
+      <c r="F3" s="78">
+        <v>0.75</v>
+      </c>
+      <c r="G3" s="78">
+        <v>0.75</v>
+      </c>
+      <c r="H3" s="78">
+        <v>0.69</v>
+      </c>
+      <c r="I3" s="78">
+        <v>0.69</v>
+      </c>
+      <c r="J3" s="78">
+        <v>0.69</v>
+      </c>
+      <c r="K3" s="78">
+        <v>0</v>
+      </c>
+      <c r="L3" s="78">
+        <v>0.62</v>
+      </c>
+      <c r="M3" s="78">
+        <v>1</v>
+      </c>
+      <c r="N3" s="78">
+        <v>1</v>
+      </c>
+      <c r="O3" s="78">
+        <v>0.94</v>
+      </c>
+      <c r="P3" s="78">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="Q3" s="78">
+        <v>0.44</v>
+      </c>
+      <c r="R3" s="78">
+        <v>0.44</v>
+      </c>
+      <c r="S3" s="79">
+        <v>0</v>
+      </c>
+      <c r="T3" s="84"/>
+      <c r="U3" s="7"/>
+      <c r="V3" s="7"/>
+      <c r="W3" s="14"/>
+    </row>
+    <row r="4" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="74"/>
+      <c r="B4" s="74"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="72"/>
+      <c r="H4" s="72"/>
+      <c r="I4" s="72"/>
+      <c r="J4" s="72"/>
+      <c r="K4" s="72"/>
+      <c r="P4" s="72"/>
+      <c r="Q4" s="72"/>
+      <c r="R4" s="72"/>
+      <c r="S4" s="72"/>
+      <c r="T4" s="72"/>
+      <c r="U4" s="72"/>
+      <c r="V4" s="72"/>
+      <c r="W4" s="72"/>
+      <c r="X4" s="72"/>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A5" s="76" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="73" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="73" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="73" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="73" t="s">
+        <v>230</v>
+      </c>
+      <c r="F5" s="73" t="s">
+        <v>231</v>
+      </c>
+      <c r="G5" s="73" t="s">
+        <v>232</v>
+      </c>
+      <c r="H5" s="73" t="s">
+        <v>233</v>
+      </c>
+      <c r="I5" s="73" t="s">
+        <v>234</v>
+      </c>
+      <c r="J5" s="73" t="s">
+        <v>235</v>
+      </c>
+      <c r="K5" s="73" t="s">
+        <v>236</v>
+      </c>
+      <c r="L5" s="73" t="s">
+        <v>237</v>
+      </c>
+      <c r="M5" s="73" t="s">
+        <v>238</v>
+      </c>
+      <c r="N5" s="73" t="s">
+        <v>244</v>
+      </c>
+      <c r="O5" s="73" t="s">
+        <v>239</v>
+      </c>
+      <c r="P5" s="73" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q5" s="73" t="s">
+        <v>241</v>
+      </c>
+      <c r="R5" s="73" t="s">
+        <v>242</v>
+      </c>
+      <c r="S5" s="71" t="s">
+        <v>243</v>
+      </c>
+      <c r="T5" s="76" t="s">
+        <v>49</v>
+      </c>
+      <c r="U5" s="73" t="s">
+        <v>142</v>
+      </c>
+      <c r="V5" s="73" t="s">
+        <v>144</v>
+      </c>
+      <c r="W5" s="73" t="s">
+        <v>227</v>
+      </c>
+      <c r="X5" s="71" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A6" s="89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B6" s="110" t="s">
+        <v>147</v>
+      </c>
+      <c r="C6" s="75" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="72">
+        <v>0.48</v>
+      </c>
+      <c r="E6" s="72">
+        <v>0.66</v>
+      </c>
+      <c r="F6" s="72">
+        <v>1</v>
+      </c>
+      <c r="G6" s="72">
+        <v>1</v>
+      </c>
+      <c r="H6" s="72">
+        <v>0.8</v>
+      </c>
+      <c r="I6" s="72">
+        <v>1</v>
+      </c>
+      <c r="J6" s="72">
+        <v>0.45</v>
+      </c>
+      <c r="K6" s="72">
+        <v>0.45</v>
+      </c>
+      <c r="L6" s="72">
+        <v>0.3</v>
+      </c>
+      <c r="M6" s="72">
+        <v>0.3</v>
+      </c>
+      <c r="N6" s="72">
+        <v>0.3</v>
+      </c>
+      <c r="O6" s="72">
+        <v>0.7</v>
+      </c>
+      <c r="P6" s="72">
+        <v>0.35</v>
+      </c>
+      <c r="Q6" s="72">
+        <v>0.45</v>
+      </c>
+      <c r="R6" s="72">
+        <v>0</v>
+      </c>
+      <c r="S6" s="77">
+        <v>0</v>
+      </c>
+      <c r="T6" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="U6" t="s">
+        <v>246</v>
+      </c>
+      <c r="V6" t="s">
+        <v>247</v>
+      </c>
+      <c r="W6" t="s">
+        <v>248</v>
+      </c>
+      <c r="X6" s="12" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="90"/>
+      <c r="B7" s="111"/>
+      <c r="C7" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="78">
+        <v>0.48</v>
+      </c>
+      <c r="E7" s="78">
+        <v>0.75</v>
+      </c>
+      <c r="F7" s="78">
+        <v>1</v>
+      </c>
+      <c r="G7" s="78">
+        <v>1</v>
+      </c>
+      <c r="H7" s="78">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="I7" s="78">
+        <v>1</v>
+      </c>
+      <c r="J7" s="78">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="K7" s="78">
+        <v>0.62</v>
+      </c>
+      <c r="L7" s="78">
+        <v>0.62</v>
+      </c>
+      <c r="M7" s="78">
+        <v>0.62</v>
+      </c>
+      <c r="N7" s="78">
+        <v>0.22</v>
+      </c>
+      <c r="O7" s="78">
+        <v>0.54</v>
+      </c>
+      <c r="P7" s="78">
+        <v>0.54</v>
+      </c>
+      <c r="Q7" s="78">
+        <v>0</v>
+      </c>
+      <c r="R7" s="78">
+        <v>0</v>
+      </c>
+      <c r="S7" s="79">
+        <v>0</v>
+      </c>
+      <c r="T7" s="84"/>
+      <c r="U7" s="7"/>
+      <c r="V7" s="7"/>
+      <c r="W7" s="7"/>
+      <c r="X7" s="14"/>
+    </row>
+    <row r="8" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="74"/>
+      <c r="B8" s="74"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="72"/>
+      <c r="H8" s="72"/>
+      <c r="I8" s="72"/>
+      <c r="J8" s="72"/>
+      <c r="K8" s="72"/>
+      <c r="L8" s="72"/>
+      <c r="M8" s="72"/>
+      <c r="P8" s="72"/>
+      <c r="Q8" s="72"/>
+      <c r="R8" s="72"/>
+      <c r="S8" s="72"/>
+      <c r="T8" s="72"/>
+      <c r="U8" s="72"/>
+      <c r="X8" s="72"/>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A9" s="76" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="73" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="73" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="73" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="73" t="s">
+        <v>263</v>
+      </c>
+      <c r="F9" s="73" t="s">
+        <v>250</v>
+      </c>
+      <c r="G9" s="73" t="s">
+        <v>251</v>
+      </c>
+      <c r="H9" s="73" t="s">
+        <v>252</v>
+      </c>
+      <c r="I9" s="73" t="s">
+        <v>253</v>
+      </c>
+      <c r="J9" s="73" t="s">
+        <v>254</v>
+      </c>
+      <c r="K9" s="73" t="s">
+        <v>255</v>
+      </c>
+      <c r="L9" s="73" t="s">
+        <v>256</v>
+      </c>
+      <c r="M9" s="73" t="s">
+        <v>257</v>
+      </c>
+      <c r="N9" s="73" t="s">
+        <v>258</v>
+      </c>
+      <c r="O9" s="73" t="s">
+        <v>266</v>
+      </c>
+      <c r="P9" s="73" t="s">
+        <v>264</v>
+      </c>
+      <c r="Q9" s="73" t="s">
+        <v>259</v>
+      </c>
+      <c r="R9" s="73" t="s">
+        <v>260</v>
+      </c>
+      <c r="S9" s="73" t="s">
+        <v>261</v>
+      </c>
+      <c r="T9" s="71" t="s">
+        <v>262</v>
+      </c>
+      <c r="U9" s="28" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A10" s="89" t="s">
+        <v>146</v>
+      </c>
+      <c r="B10" s="110" t="s">
+        <v>149</v>
+      </c>
+      <c r="C10" s="75" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="72">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="E10" s="72">
+        <v>0.39</v>
+      </c>
+      <c r="F10" s="72">
+        <v>0.9</v>
+      </c>
+      <c r="G10" s="72">
+        <v>0.9</v>
+      </c>
+      <c r="H10" s="72">
+        <v>1</v>
+      </c>
+      <c r="I10" s="72">
+        <v>0</v>
+      </c>
+      <c r="J10" s="72">
+        <v>0.1</v>
+      </c>
+      <c r="K10" s="72">
+        <v>0.1</v>
+      </c>
+      <c r="L10" s="72">
+        <v>0</v>
+      </c>
+      <c r="M10" s="72">
+        <v>0.3</v>
+      </c>
+      <c r="N10" s="72">
+        <v>0.6</v>
+      </c>
+      <c r="O10" s="72">
+        <v>0</v>
+      </c>
+      <c r="P10" s="72">
+        <v>0.18</v>
+      </c>
+      <c r="Q10" s="72">
+        <v>0.73</v>
+      </c>
+      <c r="R10" s="72">
+        <v>0</v>
+      </c>
+      <c r="S10" s="72">
+        <v>0</v>
+      </c>
+      <c r="T10" s="77">
+        <v>0</v>
+      </c>
+      <c r="U10" s="83" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="90"/>
+      <c r="B11" s="111"/>
+      <c r="C11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="78">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="E11" s="78">
+        <v>0.59</v>
+      </c>
+      <c r="F11" s="78">
+        <v>1</v>
+      </c>
+      <c r="G11" s="78">
+        <v>1</v>
+      </c>
+      <c r="H11" s="78">
+        <v>1</v>
+      </c>
+      <c r="I11" s="78">
+        <v>0.6</v>
+      </c>
+      <c r="J11" s="78">
+        <v>0.6</v>
+      </c>
+      <c r="K11" s="78">
+        <v>0.6</v>
+      </c>
+      <c r="L11" s="78">
+        <v>0</v>
+      </c>
+      <c r="M11" s="78">
+        <v>0.53</v>
+      </c>
+      <c r="N11" s="78">
+        <v>0.53</v>
+      </c>
+      <c r="O11" s="78">
+        <v>0</v>
+      </c>
+      <c r="P11" s="78">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="78">
+        <v>0</v>
+      </c>
+      <c r="R11" s="78">
+        <v>0</v>
+      </c>
+      <c r="S11" s="78">
+        <v>0</v>
+      </c>
+      <c r="T11" s="79">
+        <v>0</v>
+      </c>
+      <c r="U11" s="29"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B470A038-5A33-46E4-9DC0-73EE0BD02EB9}">
   <sheetPr>
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:P6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
@@ -2724,13 +4531,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9EAB266-A1FB-4ACC-B60E-88C7DF4D5ABD}">
   <sheetPr>
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:S3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
@@ -2812,10 +4619,10 @@
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" s="92">
+      <c r="A2" s="114">
         <v>1</v>
       </c>
-      <c r="B2" s="90" t="s">
+      <c r="B2" s="112" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="4" t="s">
@@ -2871,8 +4678,8 @@
       </c>
     </row>
     <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="93"/>
-      <c r="B3" s="91"/>
+      <c r="A3" s="115"/>
+      <c r="B3" s="113"/>
       <c r="C3" s="7" t="s">
         <v>39</v>
       </c>
@@ -2928,49 +4735,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4968849B-1DA5-49B0-87F9-037FA16ABC48}">
   <sheetPr>
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76D53979-A9C1-4366-AE84-B08F4F4C5F7F}">
-  <sheetPr>
-    <tabColor theme="3" tint="0.499984740745262"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEB907A7-035C-4DD7-877C-3D230C7BC692}">
-  <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
-  </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C60ADB6-D9A9-438B-98FC-D53C5C09C361}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76D53979-A9C1-4366-AE84-B08F4F4C5F7F}">
   <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
+    <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>